<commit_message>
feat(masterdata): TbAbility 프레임 컬럼 외부화 + dash 행 [대시 slice 2]
cast_time_ticks → startup_ticks 리네임 + active_ticks/recovery_ticks/motion_speed
컬럼 추가. dash 행(id 2: active 6, motion_speed 15, targeting Direction) 추가.
haste(id 1)는 거동 보존(active 1, motion 0).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/table/Datas/#Ability.xlsx
+++ b/table/Datas/#Ability.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K5"/>
+  <dimension ref="A1:N6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -454,22 +454,37 @@
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>cast_time_ticks</t>
+          <t>startup_ticks</t>
         </is>
       </c>
       <c r="I1" t="inlineStr">
         <is>
+          <t>active_ticks</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>recovery_ticks</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
           <t>targeting_mode</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>range</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>produces_effect_id</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>motion_speed</t>
         </is>
       </c>
     </row>
@@ -516,17 +531,32 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
+          <t>long</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
           <t>string</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr">
+      <c r="L2" t="inlineStr">
         <is>
           <t>float</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr">
+      <c r="M2" t="inlineStr">
         <is>
           <t>int</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>float</t>
         </is>
       </c>
     </row>
@@ -550,6 +580,9 @@
       <c r="I3" t="inlineStr"/>
       <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr"/>
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="inlineStr"/>
+      <c r="N3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -589,22 +622,37 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>cast_time_ticks</t>
+          <t>startup_ticks</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
+          <t>active_ticks</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>recovery_ticks</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
           <t>targeting_mode</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr">
+      <c r="L4" t="inlineStr">
         <is>
           <t>range</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr">
+      <c r="M4" t="inlineStr">
         <is>
           <t>produces_effect_id</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>motion_speed</t>
         </is>
       </c>
     </row>
@@ -637,16 +685,75 @@
       <c r="H5" t="n">
         <v>0</v>
       </c>
-      <c r="I5" t="inlineStr">
+      <c r="I5" t="n">
+        <v>1</v>
+      </c>
+      <c r="J5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K5" t="inlineStr">
         <is>
           <t>Self</t>
         </is>
       </c>
-      <c r="J5" t="n">
-        <v>0</v>
-      </c>
-      <c r="K5" t="n">
+      <c r="L5" t="n">
+        <v>0</v>
+      </c>
+      <c r="M5" t="n">
         <v>1</v>
+      </c>
+      <c r="N5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr"/>
+      <c r="B6" t="n">
+        <v>2</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>dash</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>dash</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>전방 대시</t>
+        </is>
+      </c>
+      <c r="F6" t="n">
+        <v>12</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I6" t="n">
+        <v>6</v>
+      </c>
+      <c r="J6" t="n">
+        <v>0</v>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>Direction</t>
+        </is>
+      </c>
+      <c r="L6" t="n">
+        <v>0</v>
+      </c>
+      <c r="M6" t="n">
+        <v>0</v>
+      </c>
+      <c r="N6" t="n">
+        <v>15</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat(masterdata): DamageEffect 다형 bean + attack 어빌리티 행 (B1)
__beans__에 DamageEffect{amount,range,angle} 다중필드 bean 추가(*fields 다행 연속).
#Ability.xlsx에 id=3 attack 행(startup19/active1/recovery18 ≈ 레거시 0.633s, 부채꼴 range2/angle90).
convert는 effect bean 계층 author. (B0.2 authoring 본체도 함께 박제 — 직전 커밋이 평면 source 삭제만 했음.)

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/table/Datas/#Ability.xlsx
+++ b/table/Datas/#Ability.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N6"/>
+  <dimension ref="A1:K7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -469,22 +469,7 @@
       </c>
       <c r="K1" t="inlineStr">
         <is>
-          <t>targeting_mode</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>range</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>produces_effect_id</t>
-        </is>
-      </c>
-      <c r="N1" t="inlineStr">
-        <is>
-          <t>motion_speed</t>
+          <t>effects#sep=,</t>
         </is>
       </c>
     </row>
@@ -541,22 +526,7 @@
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>string</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>float</t>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>int</t>
-        </is>
-      </c>
-      <c r="N2" t="inlineStr">
-        <is>
-          <t>float</t>
+          <t>list,AbilityEffect</t>
         </is>
       </c>
     </row>
@@ -566,23 +536,11 @@
           <t>##group</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr"/>
-      <c r="C3" t="inlineStr"/>
-      <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
           <t>c</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="inlineStr"/>
-      <c r="I3" t="inlineStr"/>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
-      <c r="L3" t="inlineStr"/>
-      <c r="M3" t="inlineStr"/>
-      <c r="N3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -637,27 +595,11 @@
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>targeting_mode</t>
-        </is>
-      </c>
-      <c r="L4" t="inlineStr">
-        <is>
-          <t>range</t>
-        </is>
-      </c>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>produces_effect_id</t>
-        </is>
-      </c>
-      <c r="N4" t="inlineStr">
-        <is>
-          <t>motion_speed</t>
+          <t>effects</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr"/>
       <c r="B5" t="n">
         <v>1</v>
       </c>
@@ -693,21 +635,11 @@
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>Self</t>
-        </is>
-      </c>
-      <c r="L5" t="n">
-        <v>0</v>
-      </c>
-      <c r="M5" t="n">
-        <v>1</v>
-      </c>
-      <c r="N5" t="n">
-        <v>0</v>
+          <t>StatusEffectApplyEffect,1</t>
+        </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr"/>
       <c r="B6" t="n">
         <v>2</v>
       </c>
@@ -736,24 +668,55 @@
         <v>0</v>
       </c>
       <c r="I6" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="J6" t="n">
         <v>0</v>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>Direction</t>
-        </is>
-      </c>
-      <c r="L6" t="n">
-        <v>0</v>
-      </c>
-      <c r="M6" t="n">
-        <v>0</v>
-      </c>
-      <c r="N6" t="n">
-        <v>15</v>
+          <t>MotionEffect,15</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" t="n">
+        <v>3</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>attack</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>attack</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>근접 공격 (부채꼴)</t>
+        </is>
+      </c>
+      <c r="F7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" t="n">
+        <v>19</v>
+      </c>
+      <c r="I7" t="n">
+        <v>1</v>
+      </c>
+      <c r="J7" t="n">
+        <v>18</v>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>DamageEffect,10,2,90</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat(masterdata): TbAbility client-only cue 컬럼 (slice 4)
attack(id3)="attack", haste/dash=빈값. 발동 연출 애니 매핑(클라 전용, group c).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/table/Datas/#Ability.xlsx
+++ b/table/Datas/#Ability.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K7"/>
+  <dimension ref="A1:L7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -469,6 +469,11 @@
       </c>
       <c r="K1" t="inlineStr">
         <is>
+          <t>cue</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
           <t>effects#sep=,</t>
         </is>
       </c>
@@ -526,6 +531,11 @@
       </c>
       <c r="K2" t="inlineStr">
         <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
           <t>list,AbilityEffect</t>
         </is>
       </c>
@@ -541,6 +551,11 @@
           <t>c</t>
         </is>
       </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -594,6 +609,11 @@
         </is>
       </c>
       <c r="K4" t="inlineStr">
+        <is>
+          <t>cue</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
         <is>
           <t>effects</t>
         </is>
@@ -633,7 +653,8 @@
       <c r="J5" t="n">
         <v>0</v>
       </c>
-      <c r="K5" t="inlineStr">
+      <c r="K5" t="inlineStr"/>
+      <c r="L5" t="inlineStr">
         <is>
           <t>StatusEffectApplyEffect,1</t>
         </is>
@@ -673,7 +694,8 @@
       <c r="J6" t="n">
         <v>0</v>
       </c>
-      <c r="K6" t="inlineStr">
+      <c r="K6" t="inlineStr"/>
+      <c r="L6" t="inlineStr">
         <is>
           <t>MotionEffect,15</t>
         </is>
@@ -714,6 +736,11 @@
         <v>18</v>
       </c>
       <c r="K7" t="inlineStr">
+        <is>
+          <t>attack</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
         <is>
           <t>DamageEffect,10,2,90</t>
         </is>

</xml_diff>

<commit_message>
feat(masterdata): attack에 KnockbackEffect 데이터 (Damage + Knockback)
Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/table/Datas/#Ability.xlsx
+++ b/table/Datas/#Ability.xlsx
@@ -653,7 +653,6 @@
       <c r="J5" t="n">
         <v>0</v>
       </c>
-      <c r="K5" t="inlineStr"/>
       <c r="L5" t="inlineStr">
         <is>
           <t>StatusEffectApplyEffect,1</t>
@@ -694,7 +693,6 @@
       <c r="J6" t="n">
         <v>0</v>
       </c>
-      <c r="K6" t="inlineStr"/>
       <c r="L6" t="inlineStr">
         <is>
           <t>MotionEffect,15</t>
@@ -742,7 +740,7 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>DamageEffect,10,2,90</t>
+          <t>DamageEffect,10,2,90,KnockbackEffect,5,2,90,12,0.8</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
data: TbAbility 이동정책 컬럼(move_scale 3 + block_jump), attack=완전정지
</commit_message>
<xml_diff>
--- a/table/Datas/#Ability.xlsx
+++ b/table/Datas/#Ability.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L7"/>
+  <dimension ref="A1:P7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -477,6 +477,26 @@
           <t>effects#sep=,</t>
         </is>
       </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>startup_move_scale</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>active_move_scale</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>recovery_move_scale</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>block_jump</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -539,6 +559,26 @@
           <t>list,AbilityEffect</t>
         </is>
       </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>bool</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -616,6 +656,26 @@
       <c r="L4" t="inlineStr">
         <is>
           <t>effects</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>startup_move_scale</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>active_move_scale</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>recovery_move_scale</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>block_jump</t>
         </is>
       </c>
     </row>
@@ -658,6 +718,20 @@
           <t>StatusEffectApplyEffect,1</t>
         </is>
       </c>
+      <c r="M5" t="n">
+        <v>1</v>
+      </c>
+      <c r="N5" t="n">
+        <v>1</v>
+      </c>
+      <c r="O5" t="n">
+        <v>1</v>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="B6" t="n">
@@ -698,6 +772,20 @@
           <t>MotionEffect,15</t>
         </is>
       </c>
+      <c r="M6" t="n">
+        <v>1</v>
+      </c>
+      <c r="N6" t="n">
+        <v>1</v>
+      </c>
+      <c r="O6" t="n">
+        <v>1</v>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="B7" t="n">
@@ -741,6 +829,20 @@
       <c r="L7" t="inlineStr">
         <is>
           <t>DamageEffect,10,2,90,KnockbackEffect,5,2,90,12,0.8</t>
+        </is>
+      </c>
+      <c r="M7" t="n">
+        <v>0</v>
+      </c>
+      <c r="N7" t="n">
+        <v>0</v>
+      </c>
+      <c r="O7" t="n">
+        <v>0</v>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>true</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(masterdata): TbCharacterLoadout + 캐릭터별 공격 어빌리티 2행
</commit_message>
<xml_diff>
--- a/table/Datas/#Ability.xlsx
+++ b/table/Datas/#Ability.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P8"/>
+  <dimension ref="A1:P10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -902,6 +902,128 @@
       <c r="P8" t="inlineStr">
         <is>
           <t>false</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>necro_attack</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>necro_attack</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>근접 공격 (부채꼴)</t>
+        </is>
+      </c>
+      <c r="F9" t="n">
+        <v>0</v>
+      </c>
+      <c r="G9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H9" t="n">
+        <v>19</v>
+      </c>
+      <c r="I9" t="n">
+        <v>1</v>
+      </c>
+      <c r="J9" t="n">
+        <v>18</v>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>attack</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>DamageEffect,10,2,90,KnockbackEffect,5,12,0.8</t>
+        </is>
+      </c>
+      <c r="M9" t="n">
+        <v>0</v>
+      </c>
+      <c r="N9" t="n">
+        <v>0</v>
+      </c>
+      <c r="O9" t="n">
+        <v>0</v>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>archer_attack</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>archer_attack</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>근접 공격 (부채꼴)</t>
+        </is>
+      </c>
+      <c r="F10" t="n">
+        <v>0</v>
+      </c>
+      <c r="G10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" t="n">
+        <v>19</v>
+      </c>
+      <c r="I10" t="n">
+        <v>1</v>
+      </c>
+      <c r="J10" t="n">
+        <v>18</v>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>attack</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>DamageEffect,10,2,90,KnockbackEffect,5,12,0.8</t>
+        </is>
+      </c>
+      <c r="M10" t="n">
+        <v>0</v>
+      </c>
+      <c r="N10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>true</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(masterdata): TbAbilityView 클라 전용 테이블 추가, Ability.cue 제거
시전 애니 이름을 어빌리티 id로 찾도록 클라 전용 뷰 테이블을 만든다.
캐릭터별로 어빌리티가 갈라진 뒤라 id 하나로 애니 스테이트가 정해진다
(3=Knight "Attack 01" / 5=Necromancer "melee attack with wand" / 6=Archer "Attack").

이름은 Animator.Play가 받는 *스테이트* 이름이다 — 트리거 파라미터 이름과 다르다.
여러 캐릭터가 함께 쓰는 global_attack(4)은 캐릭터마다 애니가 달라 행을 두지 않았다.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/table/Datas/#Ability.xlsx
+++ b/table/Datas/#Ability.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P10"/>
+  <dimension ref="A1:O10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -469,30 +469,25 @@
       </c>
       <c r="K1" t="inlineStr">
         <is>
-          <t>cue</t>
+          <t>effects#sep=,</t>
         </is>
       </c>
       <c r="L1" t="inlineStr">
         <is>
-          <t>effects#sep=,</t>
+          <t>startup_move_scale</t>
         </is>
       </c>
       <c r="M1" t="inlineStr">
         <is>
-          <t>startup_move_scale</t>
+          <t>active_move_scale</t>
         </is>
       </c>
       <c r="N1" t="inlineStr">
         <is>
-          <t>active_move_scale</t>
+          <t>recovery_move_scale</t>
         </is>
       </c>
       <c r="O1" t="inlineStr">
-        <is>
-          <t>recovery_move_scale</t>
-        </is>
-      </c>
-      <c r="P1" t="inlineStr">
         <is>
           <t>block_jump</t>
         </is>
@@ -551,12 +546,12 @@
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>string</t>
+          <t>list,AbilityEffect</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>list,AbilityEffect</t>
+          <t>float</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
@@ -570,11 +565,6 @@
         </is>
       </c>
       <c r="O2" t="inlineStr">
-        <is>
-          <t>float</t>
-        </is>
-      </c>
-      <c r="P2" t="inlineStr">
         <is>
           <t>bool</t>
         </is>
@@ -591,11 +581,6 @@
           <t>c</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>c</t>
-        </is>
-      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -650,30 +635,25 @@
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>cue</t>
+          <t>effects</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>effects</t>
+          <t>startup_move_scale</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>startup_move_scale</t>
+          <t>active_move_scale</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>active_move_scale</t>
+          <t>recovery_move_scale</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
-        <is>
-          <t>recovery_move_scale</t>
-        </is>
-      </c>
-      <c r="P4" t="inlineStr">
         <is>
           <t>block_jump</t>
         </is>
@@ -713,21 +693,21 @@
       <c r="J5" t="n">
         <v>0</v>
       </c>
-      <c r="L5" t="inlineStr">
+      <c r="K5" t="inlineStr">
         <is>
           <t>StatusEffectApplyEffect,1</t>
         </is>
       </c>
+      <c r="L5" t="n">
+        <v>1</v>
+      </c>
       <c r="M5" t="n">
         <v>1</v>
       </c>
       <c r="N5" t="n">
         <v>1</v>
       </c>
-      <c r="O5" t="n">
-        <v>1</v>
-      </c>
-      <c r="P5" t="inlineStr">
+      <c r="O5" t="inlineStr">
         <is>
           <t>false</t>
         </is>
@@ -767,21 +747,21 @@
       <c r="J6" t="n">
         <v>0</v>
       </c>
-      <c r="L6" t="inlineStr">
+      <c r="K6" t="inlineStr">
         <is>
           <t>MotionEffect,15</t>
         </is>
       </c>
+      <c r="L6" t="n">
+        <v>1</v>
+      </c>
       <c r="M6" t="n">
         <v>1</v>
       </c>
       <c r="N6" t="n">
         <v>1</v>
       </c>
-      <c r="O6" t="n">
-        <v>1</v>
-      </c>
-      <c r="P6" t="inlineStr">
+      <c r="O6" t="inlineStr">
         <is>
           <t>false</t>
         </is>
@@ -823,24 +803,19 @@
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>attack</t>
-        </is>
-      </c>
-      <c r="L7" t="inlineStr">
-        <is>
           <t>DamageEffect,10,2,90,KnockbackEffect,5,12,0.8</t>
         </is>
       </c>
+      <c r="L7" t="n">
+        <v>0</v>
+      </c>
       <c r="M7" t="n">
         <v>0</v>
       </c>
       <c r="N7" t="n">
         <v>0</v>
       </c>
-      <c r="O7" t="n">
-        <v>0</v>
-      </c>
-      <c r="P7" t="inlineStr">
+      <c r="O7" t="inlineStr">
         <is>
           <t>true</t>
         </is>
@@ -882,24 +857,19 @@
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>attack</t>
-        </is>
-      </c>
-      <c r="L8" t="inlineStr">
-        <is>
           <t>DamageEffect,30,30,360</t>
         </is>
       </c>
+      <c r="L8" t="n">
+        <v>1</v>
+      </c>
       <c r="M8" t="n">
         <v>1</v>
       </c>
       <c r="N8" t="n">
         <v>1</v>
       </c>
-      <c r="O8" t="n">
-        <v>1</v>
-      </c>
-      <c r="P8" t="inlineStr">
+      <c r="O8" t="inlineStr">
         <is>
           <t>false</t>
         </is>
@@ -943,24 +913,19 @@
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>attack</t>
-        </is>
-      </c>
-      <c r="L9" t="inlineStr">
-        <is>
           <t>DamageEffect,10,2,90,KnockbackEffect,5,12,0.8</t>
         </is>
       </c>
+      <c r="L9" t="n">
+        <v>0</v>
+      </c>
       <c r="M9" t="n">
         <v>0</v>
       </c>
       <c r="N9" t="n">
         <v>0</v>
       </c>
-      <c r="O9" t="n">
-        <v>0</v>
-      </c>
-      <c r="P9" t="inlineStr">
+      <c r="O9" t="inlineStr">
         <is>
           <t>true</t>
         </is>
@@ -1004,24 +969,19 @@
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>attack</t>
-        </is>
-      </c>
-      <c r="L10" t="inlineStr">
-        <is>
           <t>DamageEffect,10,2,90,KnockbackEffect,5,12,0.8</t>
         </is>
       </c>
+      <c r="L10" t="n">
+        <v>0</v>
+      </c>
       <c r="M10" t="n">
         <v>0</v>
       </c>
       <c r="N10" t="n">
         <v>0</v>
       </c>
-      <c r="O10" t="n">
-        <v>0</v>
-      </c>
-      <c r="P10" t="inlineStr">
+      <c r="O10" t="inlineStr">
         <is>
           <t>true</t>
         </is>

</xml_diff>